<commit_message>
add model decision tree
</commit_message>
<xml_diff>
--- a/house_price/experiments/experiments.xlsx
+++ b/house_price/experiments/experiments.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DEEP_LEARNING_SGU\house_price\experiments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SGU26_DeepLearning_Group\house_price\experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A58C35-D5F0-45A6-AB02-9A588F95D218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{086A75C9-6EB3-4DCD-A7D7-803B1C580A1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>STT</t>
   </si>
@@ -43,6 +43,15 @@
   </si>
   <si>
     <t>MAE: 15607.19</t>
+  </si>
+  <si>
+    <t>EXPER DATE</t>
+  </si>
+  <si>
+    <t>decision tree _ v1</t>
+  </si>
+  <si>
+    <t>decision tree _ v2</t>
   </si>
 </sst>
 </file>
@@ -78,11 +87,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -363,41 +374,73 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.8984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.8984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="22.9140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.9140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.4140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="1">
+      <c r="E2" s="1">
         <v>0.13413</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>46287.959027777775</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3">
+        <v>0.2094</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3">
+        <v>46287.980555555558</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4">
+        <v>0.20069999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>